<commit_message>
added sample data file
</commit_message>
<xml_diff>
--- a/part_validated.xlsx
+++ b/part_validated.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Part (FG) – Validated" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ruleset Legend" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Part (FG)-Validated" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Ruleset Legend" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -268,7 +268,7 @@
     </comment>
     <comment ref="A14" authorId="0" shapeId="0">
       <text>
-        <t>[P_RS_1] Name out of FERT range (14000000000000–14999999999999)</t>
+        <t>[P_RS_1] Name out of FERT range (14000000000000-14999999999999)</t>
       </text>
     </comment>
     <comment ref="F15" authorId="0" shapeId="0">
@@ -298,7 +298,7 @@
     </comment>
     <comment ref="A17" authorId="0" shapeId="0">
       <text>
-        <t>[P_RS_1] Name out of HAWA range (15000000000000–15999999999999)</t>
+        <t>[P_RS_1] Name out of HAWA range (15000000000000-15999999999999)</t>
       </text>
     </comment>
   </commentList>

</xml_diff>